<commit_message>
Anonymized data et sans verbatim
</commit_message>
<xml_diff>
--- a/sondage_collecte_clean.xlsx
+++ b/sondage_collecte_clean.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://014gc-my.sharepoint.com/personal/hugo_morin_hrsdc-rhdcc_gc_ca/Documents/2. Perso/Entrelacs/CCE/Matieres residuelles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://014gc-my.sharepoint.com/personal/hugo_morin_hrsdc-rhdcc_gc_ca/Documents/2. Perso/Entrelacs/CCE/Matieres residuelles/dashboard_sondage_collecte/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{E1D04663-A007-41DD-93BB-5A33B2CB81C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D4CFEC3-E1BB-486A-BEBD-2D64002AA53E}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{E1D04663-A007-41DD-93BB-5A33B2CB81C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED50E8A6-5722-4815-B1F0-0D2094566ABC}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -169,9 +169,6 @@
     <t xml:space="preserve">Ce serait bien si on pouvait avoir du composte en retour </t>
   </si>
   <si>
-    <t>.Faciliter la collecte en gardant la même  que le reste des collectes.  La gestion des bacs àdes moments différents rend le tout plus difficile.</t>
-  </si>
-  <si>
     <t>C'est dur de s'y retrouver...</t>
   </si>
   <si>
@@ -573,6 +570,9 @@
   </si>
   <si>
     <t>Est-ce que vous utiliseriez ce service de dépôt communautaire à la mairie?</t>
+  </si>
+  <si>
+    <t>Faciliter la collecte en gardant la même  que le reste des collectes.  La gestion des bacs àdes moments différents rend le tout plus difficile.</t>
   </si>
 </sst>
 </file>
@@ -953,10 +953,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
@@ -1844,7 +1844,7 @@
         <v>14</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>49</v>
+        <v>181</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>6</v>
@@ -1859,7 +1859,7 @@
         <v>12</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2" t="s">
@@ -1882,22 +1882,22 @@
         <v>8</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="2" t="s">
+      <c r="F44" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H44" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1908,13 +1908,13 @@
         <v>8</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>6</v>
@@ -1932,13 +1932,13 @@
         <v>8</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>6</v>
@@ -1987,7 +1987,7 @@
         <v>14</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2009,7 +2009,7 @@
         <v>14</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2020,22 +2020,22 @@
         <v>14</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E50" s="2" t="s">
+      <c r="F50" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2097,7 +2097,7 @@
         <v>13</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2208,7 +2208,7 @@
         <v>8</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>8</v>
@@ -2254,16 +2254,16 @@
         <v>13</v>
       </c>
       <c r="E61" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H61" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2285,7 +2285,7 @@
         <v>13</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2307,7 +2307,7 @@
         <v>14</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2324,7 +2324,7 @@
         <v>8</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>6</v>
@@ -2344,13 +2344,13 @@
         <v>8</v>
       </c>
       <c r="C65" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E65" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>6</v>
@@ -2379,7 +2379,7 @@
         <v>13</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2390,13 +2390,13 @@
         <v>8</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>7</v>
@@ -2456,22 +2456,22 @@
         <v>14</v>
       </c>
       <c r="C70" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E70" s="2" t="s">
+      <c r="F70" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H70" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2482,22 +2482,22 @@
         <v>8</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E71" s="2" t="s">
+      <c r="F71" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H71" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G71" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H71" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2552,7 +2552,7 @@
         <v>14</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>6</v>
@@ -2581,7 +2581,7 @@
         <v>13</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2616,7 +2616,7 @@
         <v>11</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>7</v>
@@ -2658,16 +2658,16 @@
         <v>11</v>
       </c>
       <c r="E79" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H79" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="F79" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H79" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2782,16 +2782,16 @@
         <v>11</v>
       </c>
       <c r="E85" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H85" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G85" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H85" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2806,7 +2806,7 @@
         <v>13</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>7</v>
@@ -2844,22 +2844,22 @@
         <v>8</v>
       </c>
       <c r="C88" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E88" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D88" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E88" s="2" t="s">
+      <c r="F88" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H88" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="F88" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G88" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H88" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2930,7 +2930,7 @@
         <v>14</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>11</v>
@@ -2993,19 +2993,19 @@
       </c>
       <c r="C95" s="2"/>
       <c r="D95" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E95" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H95" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="F95" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G95" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H95" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3047,7 +3047,7 @@
         <v>11</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3058,22 +3058,22 @@
         <v>8</v>
       </c>
       <c r="C98" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D98" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E98" s="2" t="s">
+      <c r="F98" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H98" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G98" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H98" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3115,7 +3115,7 @@
         <v>8</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3150,7 +3150,7 @@
         <v>11</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>7</v>
@@ -3179,7 +3179,7 @@
         <v>13</v>
       </c>
       <c r="H103" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3190,22 +3190,22 @@
         <v>14</v>
       </c>
       <c r="C104" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E104" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D104" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E104" s="2" t="s">
+      <c r="F104" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G104" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H104" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="F104" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G104" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H104" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="105" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3236,13 +3236,13 @@
         <v>8</v>
       </c>
       <c r="C106" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E106" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>7</v>
@@ -3271,7 +3271,7 @@
         <v>13</v>
       </c>
       <c r="H107" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="108" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3279,10 +3279,10 @@
         <v>12</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>13</v>
@@ -3330,7 +3330,7 @@
         <v>11</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>6</v>
@@ -3348,7 +3348,7 @@
         <v>8</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D111" s="2" t="s">
         <v>8</v>
@@ -3361,7 +3361,7 @@
         <v>14</v>
       </c>
       <c r="H111" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3372,22 +3372,22 @@
         <v>8</v>
       </c>
       <c r="C112" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H112" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F112" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G112" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H112" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="113" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3422,16 +3422,16 @@
         <v>8</v>
       </c>
       <c r="E114" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H114" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G114" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H114" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3446,7 +3446,7 @@
         <v>8</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F115" s="2" t="s">
         <v>6</v>
@@ -3464,22 +3464,22 @@
         <v>8</v>
       </c>
       <c r="C116" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E116" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D116" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E116" s="2" t="s">
+      <c r="F116" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H116" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G116" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H116" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3490,7 +3490,7 @@
         <v>8</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D117" s="2" t="s">
         <v>14</v>
@@ -3516,7 +3516,7 @@
         <v>8</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F118" s="2" t="s">
         <v>6</v>
@@ -3534,13 +3534,13 @@
         <v>14</v>
       </c>
       <c r="C119" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E119" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="F119" s="2" t="s">
         <v>7</v>
@@ -3582,7 +3582,7 @@
         <v>13</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F121" s="2" t="s">
         <v>6</v>
@@ -3662,22 +3662,22 @@
         <v>14</v>
       </c>
       <c r="C125" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E125" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D125" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E125" s="2" t="s">
+      <c r="F125" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H125" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="F125" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G125" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H125" s="2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3688,13 +3688,13 @@
         <v>8</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D126" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F126" s="2" t="s">
         <v>7</v>
@@ -3723,7 +3723,7 @@
         <v>13</v>
       </c>
       <c r="H127" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3745,7 +3745,7 @@
         <v>11</v>
       </c>
       <c r="H128" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3780,7 +3780,7 @@
         <v>13</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F130" s="2" t="s">
         <v>6</v>
@@ -3802,16 +3802,16 @@
         <v>13</v>
       </c>
       <c r="E131" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H131" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="F131" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G131" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H131" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3864,13 +3864,13 @@
         <v>13</v>
       </c>
       <c r="C134" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E134" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="D134" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="F134" s="2" t="s">
         <v>6</v>
@@ -3945,7 +3945,7 @@
         <v>16</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" s="2" t="s">
@@ -3968,22 +3968,22 @@
         <v>8</v>
       </c>
       <c r="C139" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E139" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="D139" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E139" s="2" t="s">
+      <c r="F139" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H139" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="F139" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G139" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H139" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3994,22 +3994,22 @@
         <v>8</v>
       </c>
       <c r="C140" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E140" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D140" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E140" s="2" t="s">
+      <c r="F140" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H140" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="F140" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G140" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H140" s="2" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4024,16 +4024,16 @@
         <v>11</v>
       </c>
       <c r="E141" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H141" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="F141" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G141" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H141" s="2" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4048,16 +4048,16 @@
         <v>14</v>
       </c>
       <c r="E142" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H142" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="F142" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G142" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H142" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4071,10 +4071,10 @@
         <v>10</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F143" s="2" t="s">
         <v>7</v>
@@ -4112,13 +4112,13 @@
         <v>14</v>
       </c>
       <c r="C145" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E145" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="D145" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E145" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="F145" s="2" t="s">
         <v>6</v>
@@ -4136,7 +4136,7 @@
         <v>8</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D146" s="2" t="s">
         <v>13</v>
@@ -4149,7 +4149,7 @@
         <v>8</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4157,10 +4157,10 @@
         <v>12</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D147" s="2" t="s">
         <v>8</v>
@@ -4253,7 +4253,7 @@
         <v>11</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4304,7 +4304,7 @@
         <v>8</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D154" s="2" t="s">
         <v>8</v>
@@ -4326,13 +4326,13 @@
         <v>8</v>
       </c>
       <c r="C155" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E155" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D155" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E155" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="F155" s="2" t="s">
         <v>6</v>
@@ -4410,13 +4410,13 @@
         <v>8</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D159" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F159" s="2" t="s">
         <v>6</v>
@@ -4434,13 +4434,13 @@
         <v>8</v>
       </c>
       <c r="C160" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E160" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="D160" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E160" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="F160" s="2" t="s">
         <v>7</v>
@@ -4478,22 +4478,22 @@
         <v>14</v>
       </c>
       <c r="C162" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E162" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="D162" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E162" s="2" t="s">
+      <c r="F162" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G162" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H162" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="F162" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G162" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H162" s="2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4504,13 +4504,13 @@
         <v>8</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D163" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F163" s="2" t="s">
         <v>7</v>
@@ -4550,13 +4550,13 @@
         <v>8</v>
       </c>
       <c r="C165" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E165" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="D165" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E165" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="F165" s="2" t="s">
         <v>6</v>
@@ -4574,22 +4574,22 @@
         <v>8</v>
       </c>
       <c r="C166" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F166" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H166" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E166" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F166" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G166" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H166" s="2" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4597,25 +4597,25 @@
         <v>12</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C167" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E167" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="D167" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E167" s="2" t="s">
+      <c r="F167" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H167" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="F167" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G167" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H167" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="168" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4650,7 +4650,7 @@
         <v>13</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F169" s="2" t="s">
         <v>6</v>
@@ -4668,7 +4668,7 @@
         <v>8</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D170" s="2" t="s">
         <v>8</v>
@@ -4681,7 +4681,7 @@
         <v>13</v>
       </c>
       <c r="H170" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4763,7 +4763,7 @@
         <v>11</v>
       </c>
       <c r="H174" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4774,22 +4774,22 @@
         <v>8</v>
       </c>
       <c r="C175" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F175" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G175" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H175" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="D175" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E175" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="F175" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G175" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H175" s="2" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="176" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4800,22 +4800,22 @@
         <v>8</v>
       </c>
       <c r="C176" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E176" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D176" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E176" s="2" t="s">
+      <c r="F176" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G176" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H176" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="F176" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G176" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H176" s="2" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4837,7 +4837,7 @@
         <v>14</v>
       </c>
       <c r="H177" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>